<commit_message>
Remove sensitive .env file
</commit_message>
<xml_diff>
--- a/reports/macro_us_report.xlsx
+++ b/reports/macro_us_report.xlsx
@@ -560,10 +560,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46023</v>
+        <v>46082</v>
       </c>
       <c r="B2" t="n">
-        <v>326.588</v>
+        <v>330.293</v>
       </c>
       <c r="C2" t="n">
         <v>4.3</v>
@@ -572,49 +572,49 @@
         <v>3.64</v>
       </c>
       <c r="E2" t="n">
-        <v>4.2135</v>
+        <v>4.245909090909091</v>
       </c>
       <c r="F2" t="n">
-        <v>0.170842649932057</v>
+        <v>0.8651438343614481</v>
       </c>
       <c r="G2" t="n">
-        <v>2.391201432150014</v>
+        <v>3.285957752865198</v>
       </c>
       <c r="H2" t="n">
-        <v>325.894</v>
+        <v>328.1136666666667</v>
       </c>
       <c r="J2" t="n">
         <v>-2.272727272727282</v>
       </c>
       <c r="K2" t="n">
-        <v>7.499999999999996</v>
+        <v>2.380952380952372</v>
       </c>
       <c r="L2" t="n">
-        <v>4.4</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="N2" t="n">
-        <v>-2.1505376344086</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
         <v>-15.93533487297921</v>
       </c>
       <c r="P2" t="n">
-        <v>3.746666666666668</v>
+        <v>3.64</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.98</v>
+        <v>3.768333333333333</v>
       </c>
       <c r="R2" t="n">
-        <v>1.697202413603938</v>
+        <v>2.911433508448447</v>
       </c>
       <c r="S2" t="n">
-        <v>-8.976957103178673</v>
+        <v>-0.8075526653788967</v>
       </c>
       <c r="T2" t="n">
-        <v>4.150190235690236</v>
+        <v>4.195066188197767</v>
       </c>
       <c r="U2" t="n">
-        <v>4.149604497354497</v>
+        <v>4.147347908913699</v>
       </c>
       <c r="V2" t="n">
         <v>1</v>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X770"/>
+  <dimension ref="A1:X772"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59827,6 +59827,150 @@
         </is>
       </c>
       <c r="X770" t="inlineStr">
+        <is>
+          <t>LOW RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B771" t="n">
+        <v>327.46</v>
+      </c>
+      <c r="C771" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D771" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="E771" t="n">
+        <v>4.12578947368421</v>
+      </c>
+      <c r="F771" t="n">
+        <v>0.267003074209704</v>
+      </c>
+      <c r="G771" t="n">
+        <v>2.434004110373222</v>
+      </c>
+      <c r="H771" t="n">
+        <v>326.693</v>
+      </c>
+      <c r="J771" t="n">
+        <v>2.325581395348841</v>
+      </c>
+      <c r="K771" t="n">
+        <v>4.761904761904767</v>
+      </c>
+      <c r="L771" t="n">
+        <v>4.366666666666666</v>
+      </c>
+      <c r="N771" t="n">
+        <v>0</v>
+      </c>
+      <c r="O771" t="n">
+        <v>-15.93533487297921</v>
+      </c>
+      <c r="P771" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="Q771" t="n">
+        <v>3.865</v>
+      </c>
+      <c r="R771" t="n">
+        <v>-2.081654831275415</v>
+      </c>
+      <c r="S771" t="n">
+        <v>-7.307555870876204</v>
+      </c>
+      <c r="T771" t="n">
+        <v>4.160823763955343</v>
+      </c>
+      <c r="U771" t="n">
+        <v>4.126442425508215</v>
+      </c>
+      <c r="V771" t="n">
+        <v>2</v>
+      </c>
+      <c r="W771" t="inlineStr">
+        <is>
+          <t>Rising Unemployment Risk; Bond Yield Stress</t>
+        </is>
+      </c>
+      <c r="X771" t="inlineStr">
+        <is>
+          <t>LOW RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B772" t="n">
+        <v>330.293</v>
+      </c>
+      <c r="C772" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D772" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="E772" t="n">
+        <v>4.245909090909091</v>
+      </c>
+      <c r="F772" t="n">
+        <v>0.8651438343614481</v>
+      </c>
+      <c r="G772" t="n">
+        <v>3.285957752865198</v>
+      </c>
+      <c r="H772" t="n">
+        <v>328.1136666666667</v>
+      </c>
+      <c r="J772" t="n">
+        <v>-2.272727272727282</v>
+      </c>
+      <c r="K772" t="n">
+        <v>2.380952380952372</v>
+      </c>
+      <c r="L772" t="n">
+        <v>4.333333333333333</v>
+      </c>
+      <c r="N772" t="n">
+        <v>0</v>
+      </c>
+      <c r="O772" t="n">
+        <v>-15.93533487297921</v>
+      </c>
+      <c r="P772" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="Q772" t="n">
+        <v>3.768333333333333</v>
+      </c>
+      <c r="R772" t="n">
+        <v>2.911433508448447</v>
+      </c>
+      <c r="S772" t="n">
+        <v>-0.8075526653788967</v>
+      </c>
+      <c r="T772" t="n">
+        <v>4.195066188197767</v>
+      </c>
+      <c r="U772" t="n">
+        <v>4.147347908913699</v>
+      </c>
+      <c r="V772" t="n">
+        <v>1</v>
+      </c>
+      <c r="W772" t="inlineStr">
+        <is>
+          <t>Bond Yield Stress</t>
+        </is>
+      </c>
+      <c r="X772" t="inlineStr">
         <is>
           <t>LOW RISK</t>
         </is>
@@ -59891,7 +60035,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-01 00:00:00</t>
+          <t>2026-03-01 00:00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -59908,7 +60052,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2.39</v>
+        <v>3.29</v>
       </c>
       <c r="F2" t="n">
         <v>4.3</v>
@@ -59917,7 +60061,7 @@
         <v>3.64</v>
       </c>
       <c r="H2" t="n">
-        <v>4.21</v>
+        <v>4.25</v>
       </c>
     </row>
   </sheetData>
@@ -59974,11 +60118,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-01-01 00:00:00</t>
+          <t>2026-03-01 00:00:00</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.39</v>
+        <v>3.29</v>
       </c>
       <c r="C2" t="n">
         <v>4.3</v>
@@ -59987,7 +60131,7 @@
         <v>3.64</v>
       </c>
       <c r="E2" t="n">
-        <v>4.21</v>
+        <v>4.25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -60001,20 +60145,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-12-01 00:00:00</t>
+          <t>2026-02-01 00:00:00</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.65</v>
+        <v>2.43</v>
       </c>
       <c r="C3" t="n">
         <v>4.4</v>
       </c>
       <c r="D3" t="n">
-        <v>3.72</v>
+        <v>3.64</v>
       </c>
       <c r="E3" t="n">
-        <v>4.14</v>
+        <v>4.13</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -60022,26 +60166,26 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-11-01 00:00:00</t>
+          <t>2026-01-01 00:00:00</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.7</v>
+        <v>2.39</v>
       </c>
       <c r="C4" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="D4" t="n">
-        <v>3.88</v>
+        <v>3.64</v>
       </c>
       <c r="E4" t="n">
-        <v>4.09</v>
+        <v>4.21</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -60055,68 +60199,68 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-10-01 00:00:00</t>
-        </is>
+          <t>2025-12-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.4</v>
       </c>
       <c r="D5" t="n">
-        <v>4.09</v>
+        <v>3.72</v>
       </c>
       <c r="E5" t="n">
-        <v>4.06</v>
+        <v>4.14</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MEDIUM RISK</t>
+          <t>LOW RISK</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-09-01 00:00:00</t>
+          <t>2025-11-01 00:00:00</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.02</v>
+        <v>2.7</v>
       </c>
       <c r="C6" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="D6" t="n">
-        <v>4.22</v>
+        <v>3.88</v>
       </c>
       <c r="E6" t="n">
-        <v>4.12</v>
+        <v>4.09</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>MEDIUM RISK</t>
+          <t>LOW RISK</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-08-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2.94</v>
-      </c>
-      <c r="C7" t="n">
-        <v>4.3</v>
+          <t>2025-10-01 00:00:00</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>4.33</v>
+        <v>4.09</v>
       </c>
       <c r="E7" t="n">
-        <v>4.26</v>
+        <v>4.06</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -60130,20 +60274,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-07-01 00:00:00</t>
+          <t>2025-09-01 00:00:00</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.74</v>
+        <v>3.02</v>
       </c>
       <c r="C8" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="D8" t="n">
-        <v>4.33</v>
+        <v>4.22</v>
       </c>
       <c r="E8" t="n">
-        <v>4.39</v>
+        <v>4.12</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -60157,20 +60301,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-06-01 00:00:00</t>
+          <t>2025-08-01 00:00:00</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.68</v>
+        <v>2.94</v>
       </c>
       <c r="C9" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="D9" t="n">
         <v>4.33</v>
       </c>
       <c r="E9" t="n">
-        <v>4.38</v>
+        <v>4.26</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -60184,11 +60328,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-07-01 00:00:00</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.38</v>
+        <v>2.74</v>
       </c>
       <c r="C10" t="n">
         <v>4.3</v>
@@ -60197,7 +60341,7 @@
         <v>4.33</v>
       </c>
       <c r="E10" t="n">
-        <v>4.42</v>
+        <v>4.39</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -60211,20 +60355,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-04-01 00:00:00</t>
+          <t>2025-06-01 00:00:00</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.33</v>
+        <v>2.68</v>
       </c>
       <c r="C11" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="D11" t="n">
         <v>4.33</v>
       </c>
       <c r="E11" t="n">
-        <v>4.28</v>
+        <v>4.38</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -60238,20 +60382,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-03-01 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2.38</v>
       </c>
       <c r="C12" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="D12" t="n">
         <v>4.33</v>
       </c>
       <c r="E12" t="n">
-        <v>4.28</v>
+        <v>4.42</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -60259,17 +60403,17 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-02-01 00:00:00</t>
+          <t>2025-04-01 00:00:00</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.8</v>
+        <v>2.33</v>
       </c>
       <c r="C13" t="n">
         <v>4.2</v>
@@ -60278,7 +60422,7 @@
         <v>4.33</v>
       </c>
       <c r="E13" t="n">
-        <v>4.45</v>
+        <v>4.28</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -60286,7 +60430,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -60327,10 +60471,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46023</v>
+        <v>46082</v>
       </c>
       <c r="B2" t="n">
-        <v>-2.312239107028653</v>
+        <v>-1.977330392967709</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -60594,19 +60738,19 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>3.034249088238892</v>
+        <v>3.038603475354307</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.7832532142796874</v>
+        <v>0.7857678672658234</v>
       </c>
       <c r="AA2" t="n">
-        <v>3.851420428121622</v>
+        <v>3.856740845161635</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.388977591799339</v>
+        <v>2.39256840776757</v>
       </c>
       <c r="AC2" t="n">
-        <v>10.05790032243954</v>
+        <v>10.07368059554934</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
@@ -60699,19 +60843,19 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>2.485250150104429</v>
+        <v>2.488987842904326</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.8997288592727748</v>
+        <v>0.9022787969393616</v>
       </c>
       <c r="AA3" t="n">
-        <v>3.555203684610881</v>
+        <v>3.560181618665561</v>
       </c>
       <c r="AB3" t="n">
-        <v>3.100984354929498</v>
+        <v>3.105214857917006</v>
       </c>
       <c r="AC3" t="n">
-        <v>10.04116704891758</v>
+        <v>10.05666311642625</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
@@ -60804,19 +60948,19 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>2.470067515835148</v>
+        <v>2.473788153876651</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.7832532142796874</v>
+        <v>0.7857678672658234</v>
       </c>
       <c r="AA4" t="n">
-        <v>3.889818894873015</v>
+        <v>3.895183707855571</v>
       </c>
       <c r="AB4" t="n">
-        <v>2.87774915038157</v>
+        <v>2.881779092545797</v>
       </c>
       <c r="AC4" t="n">
-        <v>10.02088877536942</v>
+        <v>10.03651882154384</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
@@ -60909,19 +61053,19 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>2.834561661653423</v>
+        <v>2.838691738497357</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.9579666817693184</v>
+        <v>0.9605342617761308</v>
       </c>
       <c r="AA5" t="n">
-        <v>3.900789885373413</v>
+        <v>3.906167382910981</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.29525238173632</v>
+        <v>2.298758992324265</v>
       </c>
       <c r="AC5" t="n">
-        <v>9.988570610532474</v>
+        <v>10.00415237550873</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
@@ -61014,19 +61158,19 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>3.833067311533311</v>
+        <v>3.838319016700216</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.6085397467900564</v>
+        <v>0.6110014727555162</v>
       </c>
       <c r="AA6" t="n">
-        <v>3.497605984483792</v>
+        <v>3.502517324624658</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.922678288784106</v>
+        <v>1.925850168266504</v>
       </c>
       <c r="AC6" t="n">
-        <v>9.861891331591266</v>
+        <v>9.877687982346892</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
@@ -61119,19 +61263,19 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>3.83415342959267</v>
+        <v>3.839406354803526</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.2591128118107941</v>
+        <v>0.2614686837349013</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.382410584229615</v>
+        <v>3.387188736542852</v>
       </c>
       <c r="AB7" t="n">
-        <v>2.356646112705402</v>
+        <v>2.360207881158131</v>
       </c>
       <c r="AC7" t="n">
-        <v>9.832322938338482</v>
+        <v>9.84827165623941</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
@@ -61224,19 +61368,19 @@
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>2.53818027324209</v>
+        <v>2.541977422816475</v>
       </c>
       <c r="Z8" t="n">
-        <v>1.016204504265862</v>
+        <v>1.0187897266129</v>
       </c>
       <c r="AA8" t="n">
-        <v>3.020367897716485</v>
+        <v>3.024727459714316</v>
       </c>
       <c r="AB8" t="n">
-        <v>3.232519208615237</v>
+        <v>3.236867886236529</v>
       </c>
       <c r="AC8" t="n">
-        <v>9.807271883839674</v>
+        <v>9.82236249538022</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
@@ -61329,19 +61473,19 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>2.1188505019269</v>
+        <v>2.122176615460348</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.9579666817693184</v>
+        <v>0.9605342617761308</v>
       </c>
       <c r="AA9" t="n">
-        <v>3.747196018367843</v>
+        <v>3.752395932135239</v>
       </c>
       <c r="AB9" t="n">
-        <v>2.816038068752285</v>
+        <v>2.820012567934917</v>
       </c>
       <c r="AC9" t="n">
-        <v>9.640051270816343</v>
+        <v>9.655119377306637</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
@@ -61434,19 +61578,19 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>2.084921458031143</v>
+        <v>2.088209458834223</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.9579666817693184</v>
+        <v>0.9605342617761308</v>
       </c>
       <c r="AA10" t="n">
-        <v>3.906275380623612</v>
+        <v>3.911659220438687</v>
       </c>
       <c r="AB10" t="n">
-        <v>2.602670187168096</v>
+        <v>2.606452990609553</v>
       </c>
       <c r="AC10" t="n">
-        <v>9.55183370759217</v>
+        <v>9.566855931658592</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
@@ -61539,19 +61683,19 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>2.29023417180821</v>
+        <v>2.293752801806895</v>
       </c>
       <c r="Z11" t="n">
-        <v>1.190917971755493</v>
+        <v>1.193556121123207</v>
       </c>
       <c r="AA11" t="n">
-        <v>2.803690835333628</v>
+        <v>2.807799877369966</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.172745365006817</v>
+        <v>3.177040340115958</v>
       </c>
       <c r="AC11" t="n">
-        <v>9.457588343904147</v>
+        <v>9.472149140416027</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
@@ -61815,19 +61959,19 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>-0.8462190948353623</v>
+        <v>-0.846223664548133</v>
       </c>
       <c r="Z2" t="n">
-        <v>-0.8474058156235353</v>
+        <v>-0.8453851481637114</v>
       </c>
       <c r="AA2" t="n">
-        <v>-1.154093987684894</v>
+        <v>-1.154560898869245</v>
       </c>
       <c r="AB2" t="n">
-        <v>-1.684324897201521</v>
+        <v>-1.684393651426613</v>
       </c>
       <c r="AC2" t="n">
-        <v>-4.532043795345313</v>
+        <v>-4.530563363007703</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
@@ -61915,19 +62059,19 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>-1.376922307632644</v>
+        <v>-1.377523019945746</v>
       </c>
       <c r="Z3" t="n">
-        <v>-0.4979788806442735</v>
+        <v>-0.4958523591430969</v>
       </c>
       <c r="AA3" t="n">
-        <v>-1.293974116564967</v>
+        <v>-1.294602755825724</v>
       </c>
       <c r="AB3" t="n">
-        <v>-1.241123715324452</v>
+        <v>-1.240794285069207</v>
       </c>
       <c r="AC3" t="n">
-        <v>-4.409999020166337</v>
+        <v>-4.408772419983774</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
@@ -62015,19 +62159,19 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>-1.334481115998588</v>
+        <v>-1.335034153826721</v>
       </c>
       <c r="Z4" t="n">
-        <v>-0.4979788806442735</v>
+        <v>-0.4958523591430969</v>
       </c>
       <c r="AA4" t="n">
-        <v>-1.299459611815166</v>
+        <v>-1.300094593353429</v>
       </c>
       <c r="AB4" t="n">
-        <v>-1.276113282314748</v>
+        <v>-1.275815287676371</v>
       </c>
       <c r="AC4" t="n">
-        <v>-4.408032890772775</v>
+        <v>-4.406796393999618</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
@@ -62115,19 +62259,19 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>-1.069791181548276</v>
+        <v>-1.070046891336932</v>
       </c>
       <c r="Z5" t="n">
-        <v>-0.6144545256373609</v>
+        <v>-0.6123632888166353</v>
       </c>
       <c r="AA5" t="n">
-        <v>-1.225405425937481</v>
+        <v>-1.225954786729411</v>
       </c>
       <c r="AB5" t="n">
-        <v>-1.468653094003009</v>
+        <v>-1.468528082578568</v>
       </c>
       <c r="AC5" t="n">
-        <v>-4.378304227126126</v>
+        <v>-4.376893049461547</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
@@ -62215,19 +62359,19 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>-0.7781631169376881</v>
+        <v>-0.7780912388983938</v>
       </c>
       <c r="Z6" t="n">
-        <v>-1.371546218092428</v>
+        <v>-1.369684331694633</v>
       </c>
       <c r="AA6" t="n">
-        <v>-0.7728520677960694</v>
+        <v>-0.7728781906937422</v>
       </c>
       <c r="AB6" t="n">
-        <v>-1.402148618411039</v>
+        <v>-1.401963857484258</v>
       </c>
       <c r="AC6" t="n">
-        <v>-4.324710021237225</v>
+        <v>-4.322617618771028</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
@@ -62243,76 +62387,71 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2019-10-01</t>
+          <t>2015-04-01</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>257.155</v>
+        <v>236.222</v>
       </c>
       <c r="C7" t="n">
-        <v>3.6</v>
+        <v>5.4</v>
       </c>
       <c r="D7" t="n">
-        <v>1.83</v>
+        <v>0.12</v>
       </c>
       <c r="E7" t="n">
-        <v>1.706818181818182</v>
+        <v>1.935</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2827282299262768</v>
+        <v>0.1042478896158938</v>
       </c>
       <c r="G7" t="n">
-        <v>1.73397369961863</v>
+        <v>-0.1040309893939106</v>
       </c>
       <c r="H7" t="n">
-        <v>256.5403333333333</v>
+        <v>235.8466666666667</v>
       </c>
       <c r="I7" t="n">
-        <v>255.9886666666666</v>
+        <v>235.9203333333333</v>
       </c>
       <c r="J7" t="n">
-        <v>2.857142857142869</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>-5.263157894736836</v>
+        <v>-12.90322580645161</v>
       </c>
       <c r="L7" t="n">
-        <v>3.566666666666666</v>
+        <v>5.433333333333334</v>
       </c>
       <c r="M7" t="n">
-        <v>3.6</v>
+        <v>5.566666666666666</v>
       </c>
       <c r="N7" t="n">
-        <v>-10.29411764705882</v>
+        <v>9.090909090909085</v>
       </c>
       <c r="O7" t="n">
-        <v>-16.43835616438356</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="P7" t="n">
-        <v>2</v>
+        <v>0.1133333333333336</v>
       </c>
       <c r="Q7" t="n">
-        <v>2.195</v>
+        <v>0.11</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4306079328144641</v>
+        <v>-5.273698264352456</v>
       </c>
       <c r="S7" t="n">
-        <v>-45.85436193222783</v>
+        <v>-28.47209998239746</v>
       </c>
       <c r="T7" t="n">
-        <v>1.677560606060607</v>
+        <v>1.98433014354067</v>
       </c>
       <c r="U7" t="n">
-        <v>1.926795454545454</v>
+        <v>2.061219785575049</v>
       </c>
       <c r="V7" t="n">
-        <v>1</v>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>Rising Unemployment Risk</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -62320,19 +62459,19 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>-0.7604839337967301</v>
+        <v>-1.417901405651566</v>
       </c>
       <c r="Z7" t="n">
-        <v>-1.313308395595885</v>
+        <v>-0.2628304997960203</v>
       </c>
       <c r="AA7" t="n">
-        <v>-0.8304497679231581</v>
+        <v>-1.300094593353429</v>
       </c>
       <c r="AB7" t="n">
-        <v>-1.399659146062676</v>
+        <v>-1.321780353598273</v>
       </c>
       <c r="AC7" t="n">
-        <v>-4.30390124337845</v>
+        <v>-4.302606852399288</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
@@ -62348,71 +62487,76 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2015-04-01</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>236.222</v>
+        <v>257.155</v>
       </c>
       <c r="C8" t="n">
-        <v>5.4</v>
+        <v>3.6</v>
       </c>
       <c r="D8" t="n">
-        <v>0.12</v>
+        <v>1.83</v>
       </c>
       <c r="E8" t="n">
-        <v>1.935</v>
+        <v>1.706818181818182</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1042478896158938</v>
+        <v>0.2827282299262768</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.1040309893939106</v>
+        <v>1.73397369961863</v>
       </c>
       <c r="H8" t="n">
-        <v>235.8466666666667</v>
+        <v>256.5403333333333</v>
       </c>
       <c r="I8" t="n">
-        <v>235.9203333333333</v>
+        <v>255.9886666666666</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>2.857142857142869</v>
       </c>
       <c r="K8" t="n">
-        <v>-12.90322580645161</v>
+        <v>-5.263157894736836</v>
       </c>
       <c r="L8" t="n">
-        <v>5.433333333333334</v>
+        <v>3.566666666666666</v>
       </c>
       <c r="M8" t="n">
-        <v>5.566666666666666</v>
+        <v>3.6</v>
       </c>
       <c r="N8" t="n">
-        <v>9.090909090909085</v>
+        <v>-10.29411764705882</v>
       </c>
       <c r="O8" t="n">
-        <v>33.33333333333333</v>
+        <v>-16.43835616438356</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1133333333333336</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.11</v>
+        <v>2.195</v>
       </c>
       <c r="R8" t="n">
-        <v>-5.273698264352456</v>
+        <v>0.4306079328144641</v>
       </c>
       <c r="S8" t="n">
-        <v>-28.47209998239746</v>
+        <v>-45.85436193222783</v>
       </c>
       <c r="T8" t="n">
-        <v>1.98433014354067</v>
+        <v>1.677560606060607</v>
       </c>
       <c r="U8" t="n">
-        <v>2.061219785575049</v>
+        <v>1.926795454545454</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Rising Unemployment Risk</t>
+        </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -62420,19 +62564,19 @@
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>-1.417255386910727</v>
+        <v>-0.760392196608376</v>
       </c>
       <c r="Z8" t="n">
-        <v>-0.2650275906580986</v>
+        <v>-1.311428866857864</v>
       </c>
       <c r="AA8" t="n">
-        <v>-1.299459611815166</v>
+        <v>-0.8305424847346454</v>
       </c>
       <c r="AB8" t="n">
-        <v>-1.322037088989509</v>
+        <v>-1.399472148523508</v>
       </c>
       <c r="AC8" t="n">
-        <v>-4.3037796783735</v>
+        <v>-4.301835696724394</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
@@ -62520,19 +62664,19 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>-0.543462979503073</v>
+        <v>-0.543127461171324</v>
       </c>
       <c r="Z9" t="n">
-        <v>-1.371546218092428</v>
+        <v>-1.369684331694633</v>
       </c>
       <c r="AA9" t="n">
-        <v>-0.8990184585506447</v>
+        <v>-0.8991904538309589</v>
       </c>
       <c r="AB9" t="n">
-        <v>-1.468581477930222</v>
+        <v>-1.468456402163875</v>
       </c>
       <c r="AC9" t="n">
-        <v>-4.282609134076368</v>
+        <v>-4.280458648860792</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
@@ -62620,19 +62764,19 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>-1.293857426157755</v>
+        <v>-1.29436483111329</v>
       </c>
       <c r="Z10" t="n">
-        <v>-0.43974105814773</v>
+        <v>-0.437596894306328</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1.293974116564967</v>
+        <v>-1.294602755825724</v>
       </c>
       <c r="AB10" t="n">
-        <v>-1.243067580157247</v>
+        <v>-1.24273989632516</v>
       </c>
       <c r="AC10" t="n">
-        <v>-4.270640181027699</v>
+        <v>-4.269304377570502</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
@@ -62720,19 +62864,19 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>-0.7591734275859935</v>
+        <v>-0.7590802182969223</v>
       </c>
       <c r="Z11" t="n">
-        <v>-1.313308395595885</v>
+        <v>-1.311428866857864</v>
       </c>
       <c r="AA11" t="n">
-        <v>-0.7481673391701743</v>
+        <v>-0.7481649218190694</v>
       </c>
       <c r="AB11" t="n">
-        <v>-1.427027879333494</v>
+        <v>-1.426865470638581</v>
       </c>
       <c r="AC11" t="n">
-        <v>-4.247677041685547</v>
+        <v>-4.245539477612438</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>

</xml_diff>